<commit_message>
feat: import HBM4 mass-production news article (news-article template)
Add the second news article (samsung-ships-industry-first-commercial-hbm4)
using the existing news-article template — no new blocks or infrastructure,
content imported via the shared parsers/transformers/import script.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-news-article.report.xlsx
+++ b/tools/importer/reports/import-news-article.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
   <si>
     <t>_reportFile</t>
   </si>
@@ -80,6 +80,21 @@
   </si>
   <si>
     <t>https://semiconductor.samsung.com/kr/news-events/news/samsung-electronics-begins-shipment-of-industry-first-hbm4e-samples/</t>
+  </si>
+  <si>
+    <t>kr/news-events/news/samsung-ships-industry-first-commercial-hbm4-with-ultimate-performance-for-ai-computing.report.json</t>
+  </si>
+  <si>
+    <t>kr/news-events/news/samsung-ships-industry-first-commercial-hbm4-with-ultimate-performance-for-ai-computing</t>
+  </si>
+  <si>
+    <t>2026-06-29T02:39:45.473Z</t>
+  </si>
+  <si>
+    <t>삼성전자, 세계 최초 업계 최고 성능의 HBM4 양산 출하 | 삼성반도체</t>
+  </si>
+  <si>
+    <t>https://semiconductor.samsung.com/kr/news-events/news/samsung-ships-industry-first-commercial-hbm4-with-ultimate-performance-for-ai-computing/</t>
   </si>
 </sst>
 </file>
@@ -468,13 +483,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="37" customWidth="1"/>
+    <col min="7" max="7" width="42" customWidth="1"/>
     <col min="8" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
@@ -554,6 +569,32 @@
       </c>
       <c r="H3" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: import SSD virtualization tech-blog (news-article template)
Add the tech-blog article (a-peek-into-ssd-virtualization) via the existing
news-article template. The newsroom-banner block is absent on this article
(optional block, gracefully skipped) — no infrastructure changes needed.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-news-article.report.xlsx
+++ b/tools/importer/reports/import-news-article.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
   <si>
     <t>_reportFile</t>
   </si>
@@ -95,6 +95,24 @@
   </si>
   <si>
     <t>https://semiconductor.samsung.com/kr/news-events/news/samsung-ships-industry-first-commercial-hbm4-with-ultimate-performance-for-ai-computing/</t>
+  </si>
+  <si>
+    <t>kr/news-events/tech-blog/a-peek-into-ssd-virtualization.report.json</t>
+  </si>
+  <si>
+    <t>["article-header","article-image","tags-hashtag","tags-hashtag","cards-news"]</t>
+  </si>
+  <si>
+    <t>kr/news-events/tech-blog/a-peek-into-ssd-virtualization</t>
+  </si>
+  <si>
+    <t>2026-06-29T02:43:22.977Z</t>
+  </si>
+  <si>
+    <t>SSD 가상화 기술이 바꾸는 차세대 시스템 아키텍처 | 삼성반도체</t>
+  </si>
+  <si>
+    <t>https://semiconductor.samsung.com/kr/news-events/tech-blog/a-peek-into-ssd-virtualization/</t>
   </si>
 </sst>
 </file>
@@ -483,7 +501,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -597,6 +615,32 @@
         <v>27</v>
       </c>
     </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: keep article footnote/trademark lines on one line
Flatten <sup> elements inside the news-article rich-text body in
beforeTransform, so html2md no longer splits a sentence containing an
inline superscript (e.g. "* NVM Express® 및 NVMe®는 …상표입니다.") across
multiple paragraphs. Re-imported all three news-article pages.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-news-article.report.xlsx
+++ b/tools/importer/reports/import-news-article.report.xlsx
@@ -73,7 +73,7 @@
     <t>news-article</t>
   </si>
   <si>
-    <t>2026-06-28T17:27:12.251Z</t>
+    <t>2026-06-29T02:50:23.205Z</t>
   </si>
   <si>
     <t>삼성전자, 세계 최초 HBM4E 12단 샘플 출하 | 삼성반도체</t>
@@ -88,7 +88,7 @@
     <t>kr/news-events/news/samsung-ships-industry-first-commercial-hbm4-with-ultimate-performance-for-ai-computing</t>
   </si>
   <si>
-    <t>2026-06-29T02:39:45.473Z</t>
+    <t>2026-06-29T02:50:31.855Z</t>
   </si>
   <si>
     <t>삼성전자, 세계 최초 업계 최고 성능의 HBM4 양산 출하 | 삼성반도체</t>
@@ -106,7 +106,7 @@
     <t>kr/news-events/tech-blog/a-peek-into-ssd-virtualization</t>
   </si>
   <si>
-    <t>2026-06-29T02:43:22.977Z</t>
+    <t>2026-06-29T02:49:35.717Z</t>
   </si>
   <si>
     <t>SSD 가상화 기술이 바꾸는 차세대 시스템 아키텍처 | 삼성반도체</t>

</xml_diff>

<commit_message>
feat: import COMPUTEX 2026 tech-blog (news-article template)
Add the COMPUTEX 2026 tech-blog article via the existing news-article
template — content-only import, no infrastructure changes.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-news-article.report.xlsx
+++ b/tools/importer/reports/import-news-article.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
   <si>
     <t>_reportFile</t>
   </si>
@@ -113,6 +113,24 @@
   </si>
   <si>
     <t>https://semiconductor.samsung.com/kr/news-events/tech-blog/a-peek-into-ssd-virtualization/</t>
+  </si>
+  <si>
+    <t>kr/news-events/tech-blog/samsung-showcases-next-generationa-ai-semiconductor-innovations-at-computex-2026.report.json</t>
+  </si>
+  <si>
+    <t>["article-header","article-image","article-image","article-image","tags-hashtag","tags-hashtag","cards-news"]</t>
+  </si>
+  <si>
+    <t>kr/news-events/tech-blog/samsung-showcases-next-generationa-ai-semiconductor-innovations-at-computex-2026</t>
+  </si>
+  <si>
+    <t>2026-06-29T02:52:21.869Z</t>
+  </si>
+  <si>
+    <t>삼성전자, COMPUTEX 2026에서 AI 시대 반도체 경쟁력의 새로운 기준을 제시하다. | 삼성반도체</t>
+  </si>
+  <si>
+    <t>https://semiconductor.samsung.com/kr/news-events/tech-blog/samsung-showcases-next-generationa-ai-semiconductor-innovations-at-computex-2026/</t>
   </si>
 </sst>
 </file>
@@ -501,14 +519,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="42" customWidth="1"/>
-    <col min="8" max="8" width="50" customWidth="1"/>
+    <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -639,6 +656,32 @@
       </c>
       <c r="H5" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>